<commit_message>
Update ETF PE history and report
</commit_message>
<xml_diff>
--- a/etf_analyst_target_outputs/ETF_PE_history.xlsx
+++ b/etf_analyst_target_outputs/ETF_PE_history.xlsx
@@ -434,10 +434,10 @@
         <v>8</v>
       </c>
       <c r="C2">
-        <v>53.32705710313409</v>
+        <v>53.26449181340857</v>
       </c>
       <c r="D2">
-        <v>25.97299879241849</v>
+        <v>25.93249319663132</v>
       </c>
       <c r="E2">
         <v>0.9262</v>
@@ -446,7 +446,7 @@
         <v>0.9262</v>
       </c>
       <c r="G2">
-        <v>0.3872030958911865</v>
+        <v>0.3892839481608621</v>
       </c>
       <c r="H2">
         <v>0.9262</v>
@@ -460,10 +460,10 @@
         <v>9</v>
       </c>
       <c r="C3">
-        <v>34.53148244944686</v>
+        <v>34.42170829708593</v>
       </c>
       <c r="D3">
-        <v>26.08589601670652</v>
+        <v>26.01477334208454</v>
       </c>
       <c r="E3">
         <v>0.9984</v>
@@ -472,7 +472,7 @@
         <v>0.9984</v>
       </c>
       <c r="G3">
-        <v>0.06748132491122871</v>
+        <v>0.06472843849581267</v>
       </c>
       <c r="H3">
         <v>0.9984</v>
@@ -486,10 +486,10 @@
         <v>10</v>
       </c>
       <c r="C4">
-        <v>36.61274523339704</v>
+        <v>36.56347931591439</v>
       </c>
       <c r="D4">
-        <v>22.73265684308589</v>
+        <v>22.72964238966481</v>
       </c>
       <c r="E4">
         <v>0.9990740999999999</v>
@@ -498,7 +498,7 @@
         <v>0.9990740999999999</v>
       </c>
       <c r="G4">
-        <v>0.1662814267095185</v>
+        <v>0.1650893258330652</v>
       </c>
       <c r="H4">
         <v>0.9990740999999999</v>
@@ -512,10 +512,10 @@
         <v>11</v>
       </c>
       <c r="C5">
-        <v>54.62492179530582</v>
+        <v>54.66910192050099</v>
       </c>
       <c r="D5">
-        <v>22.52323336195511</v>
+        <v>22.56574131784717</v>
       </c>
       <c r="E5">
         <v>0.9999</v>
@@ -524,7 +524,7 @@
         <v>0.9999</v>
       </c>
       <c r="G5">
-        <v>0.545673771411969</v>
+        <v>0.5446150983617628</v>
       </c>
       <c r="H5">
         <v>0.9999</v>
@@ -538,10 +538,10 @@
         <v>12</v>
       </c>
       <c r="C6">
-        <v>57.12305147755242</v>
+        <v>57.16392578808276</v>
       </c>
       <c r="D6">
-        <v>23.53933454639179</v>
+        <v>23.58706076165031</v>
       </c>
       <c r="E6">
         <v>0.9991</v>
@@ -550,7 +550,7 @@
         <v>0.9991</v>
       </c>
       <c r="G6">
-        <v>0.6981350019688173</v>
+        <v>0.6983902424541246</v>
       </c>
       <c r="H6">
         <v>0.9991</v>
@@ -564,10 +564,10 @@
         <v>13</v>
       </c>
       <c r="C7">
-        <v>35.88867319884837</v>
+        <v>35.91957141339604</v>
       </c>
       <c r="D7">
-        <v>19.04521398750263</v>
+        <v>19.10923935143763</v>
       </c>
       <c r="E7">
         <v>0.9996491399999999</v>
@@ -576,7 +576,7 @@
         <v>0.9996491399999999</v>
       </c>
       <c r="G7">
-        <v>0.2277471697384601</v>
+        <v>0.2290872260284964</v>
       </c>
       <c r="H7">
         <v>0.9985614899999999</v>
@@ -590,10 +590,10 @@
         <v>14</v>
       </c>
       <c r="C8">
-        <v>28.22738048024621</v>
+        <v>28.13794731775636</v>
       </c>
       <c r="D8">
-        <v>23.67423393518881</v>
+        <v>23.59847768192577</v>
       </c>
       <c r="E8">
         <v>0.9997295369999999</v>
@@ -602,7 +602,7 @@
         <v>0.9997295369999999</v>
       </c>
       <c r="G8">
-        <v>0.03956039626956498</v>
+        <v>0.03662381108768376</v>
       </c>
       <c r="H8">
         <v>0.9997295369999999</v>
@@ -616,10 +616,10 @@
         <v>15</v>
       </c>
       <c r="C9">
-        <v>40.71619570965345</v>
+        <v>40.69797668816307</v>
       </c>
       <c r="D9">
-        <v>21.56447268795337</v>
+        <v>21.57531855713585</v>
       </c>
       <c r="E9">
         <v>0.99909852</v>
@@ -628,7 +628,7 @@
         <v>0.99909852</v>
       </c>
       <c r="G9">
-        <v>0.2359075884948187</v>
+        <v>0.2353178647851411</v>
       </c>
       <c r="H9">
         <v>0.9974930900000001</v>

</xml_diff>